<commit_message>
Z3: get better witnesses
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -824,6 +824,370 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A * A^-1 = I</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>7.905498743057251</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>(A^-1)^-1 = A</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" t="n">
+        <v>33.27820491790771</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>(A*B)^-1 = B^-1 * A^-1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>335.6147589683533</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>(A*B*C)^-1 = C^-1 * B^-1 * A^-1</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>1800.611073970795</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>A(BC) = (AB)C</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>29.41067790985107</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>det(A*B) = det(A) * det(B)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>7.315605401992798</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>det(A^-1) = 1/det(A)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>6.153125286102295</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>A(B+C) = AB + AC</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>7.704192876815796</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>(A+B)^T = A^T + B^T</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>UNSAT</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>2</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.0001485347747802734</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>(A*B)^T = B^T * A^T</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>UNSAT</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2</v>
+      </c>
+      <c r="D25" t="n">
+        <v>861.3670892715454</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>(A^T)^-1 = (A^-1)^T</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1800.637891054153</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>tr(A + B) = tr(A) + tr(B)</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" t="n">
+        <v>4.091246843338013</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>tr(AB) = tr(BA)</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" t="n">
+        <v>1.446502208709717</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>det(kA) = k^n * det(A)</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>3.354055166244507</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update Z3 values with N=3
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1188,6 +1188,84 @@
         <v>0</v>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>A(BC) = (AB)C</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" t="n">
+        <v>238.0667943954468</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>A(B+C) = AB + AC</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" t="n">
+        <v>345.9960956573486</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>det(kA) = k^n * det(A)</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>SAT</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" t="n">
+        <v>153.9955432415009</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>